<commit_message>
Fix: use enumarate to check row index
</commit_message>
<xml_diff>
--- a/Student_analysis_26.0.xlsx
+++ b/Student_analysis_26.0.xlsx
@@ -465,11 +465,7 @@
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Wilson sossion</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Algebra</t>
@@ -488,11 +484,7 @@
       <c r="A4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Wilson sossion</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Measurement</t>
@@ -511,11 +503,7 @@
       <c r="A5" t="n">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Wilson sossion</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Geomentry</t>
@@ -534,11 +522,7 @@
       <c r="A6" t="n">
         <v>4</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Wilson sossion</t>
-        </is>
-      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Data Handling and Probability</t>

</xml_diff>